<commit_message>
FOVI 2026: formulario v0.4 con nuevo título y regiones abiertas; presupuesto/Gantt y notas actualizados
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4g3Yf3jcPuX77QSmk15pC
</commit_message>
<xml_diff>
--- a/fovi2026/FOVI2026_Presupuesto-carta-gantt_v0.1.xlsx
+++ b/fovi2026/FOVI2026_Presupuesto-carta-gantt_v0.1.xlsx
@@ -2191,7 +2191,7 @@
       <c r="C5" s="184" t="n"/>
       <c r="D5" s="186" t="inlineStr">
         <is>
-          <t>Red INTEEGRA-Saúde: salud, territorio y sustentabilidad en la atención primaria. Vinculación entre Santiago y el Maule con Angola, Portugal y Brasil</t>
+          <t>INTEEGRA-Saúde: salud, territorio y sustentabilidad en la atención primaria</t>
         </is>
       </c>
       <c r="E5" s="183" t="n"/>
@@ -2777,7 +2777,7 @@
       <c r="B21" s="192" t="n"/>
       <c r="C21" s="190" t="inlineStr">
         <is>
-          <t>2.4 Análisis geoespacial Santiago–Maule; datos de Luanda; caso documental Ceará</t>
+          <t>2.4 Análisis geoespacial Santiago y regiones asociadas; datos de Luanda; caso documental Ceará</t>
         </is>
       </c>
       <c r="D21" s="191" t="inlineStr">
@@ -2981,7 +2981,7 @@
       <c r="B27" s="192" t="n"/>
       <c r="C27" s="190" t="inlineStr">
         <is>
-          <t>3.3 Visita de investigadores IPC y UJPA: ponencias en Santiago y jornada en el Maule</t>
+          <t>3.3 Visita de investigadores IPC y UJPA: ponencias en Santiago y jornada en una región asociada</t>
         </is>
       </c>
       <c r="D27" s="191" t="inlineStr">
@@ -4566,8 +4566,8 @@
     <mergeCell ref="C9:C10"/>
     <mergeCell ref="B9:B10"/>
     <mergeCell ref="D9:D10"/>
+    <mergeCell ref="B32:B38"/>
     <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B32:B38"/>
     <mergeCell ref="B18:B24"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B25:B31"/>
@@ -4697,7 +4697,7 @@
       </c>
       <c r="D8" s="200" t="inlineStr">
         <is>
-          <t>Red INTEEGRA-Saúde: salud, territorio y sustentabilidad en la atención primaria. Vinculación entre Santiago y el Maule con Angola, Portugal y Brasil</t>
+          <t>INTEEGRA-Saúde: salud, territorio y sustentabilidad en la atención primaria</t>
         </is>
       </c>
       <c r="E8" s="201" t="n"/>
@@ -5506,7 +5506,6 @@
     <mergeCell ref="D6:H6"/>
     <mergeCell ref="D8:H8"/>
     <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D20:D21"/>
     <mergeCell ref="D10:H10"/>
     <mergeCell ref="C5:H5"/>
     <mergeCell ref="D38:E38"/>
@@ -5515,8 +5514,9 @@
     <mergeCell ref="C40:D40"/>
     <mergeCell ref="C23:C30"/>
     <mergeCell ref="D14:D19"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="C3:H4"/>
     <mergeCell ref="F12:H12"/>
-    <mergeCell ref="C3:H4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" scale="80"/>
@@ -6135,7 +6135,7 @@
       </c>
       <c r="D29" s="236" t="inlineStr">
         <is>
-          <t>Software SIG, datos y licencias para el protocolo común y el análisis geoespacial del estudio comparado (Santiago, Maule, Luanda, centro de Portugal). ESTIMACIÓN.</t>
+          <t>Software SIG, datos y licencias para el protocolo común y el análisis geoespacial del estudio comparado (Santiago, regiones asociadas, Luanda, centro de Portugal). ESTIMACIÓN.</t>
         </is>
       </c>
       <c r="H29" s="231" t="n"/>
@@ -7739,7 +7739,7 @@
       </c>
       <c r="D20" s="235" t="inlineStr">
         <is>
-          <t>Visita a Chile de un/a investigador/a del IPC (Portugal) para ponencias y taller en Santiago y el Maule: pasaje aéreo económico ida y vuelta. ESTIMACIÓN: cotizar.</t>
+          <t>Visita a Chile de un/a investigador/a del IPC (Portugal) para ponencias y taller en Santiago y una región asociada: pasaje aéreo económico ida y vuelta. ESTIMACIÓN: cotizar.</t>
         </is>
       </c>
     </row>
@@ -7769,7 +7769,7 @@
       </c>
       <c r="D22" s="236" t="inlineStr">
         <is>
-          <t>2 investigadores/as extranjeros/as × 8 días × $150.000 por día (tope de viático nacional $150.000/día; máximo 10 días). Alojamiento y manutención en Santiago y el Maule.</t>
+          <t>2 investigadores/as extranjeros/as × 8 días × $150.000 por día (tope de viático nacional $150.000/día; máximo 10 días). Alojamiento y manutención en Santiago y una región asociada.</t>
         </is>
       </c>
     </row>
@@ -7799,7 +7799,7 @@
       </c>
       <c r="D24" s="236" t="inlineStr">
         <is>
-          <t>Traslado terrestre Santiago–Maule (ida y vuelta) para la jornada territorial. ESTIMACIÓN.</t>
+          <t>Traslado terrestre a la región asociada (ida y vuelta) para la jornada territorial. ESTIMACIÓN: ajustar según destino (con Biobío probablemente sube).</t>
         </is>
       </c>
     </row>
@@ -7829,7 +7829,7 @@
       </c>
       <c r="D26" s="236" t="inlineStr">
         <is>
-          <t>Taller presencial en Santiago y jornada territorial en el Maule con la UCM: arriendo de sala, materiales y difusión. No incluye alimentación ni honorarios de organización.</t>
+          <t>Taller presencial en Santiago y jornada territorial en una región asociada con las instituciones nacionales asociadas: arriendo de sala, materiales y difusión. No incluye alimentación ni honorarios de organización.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FOVI 2026: actividades calzadas con el presupuesto y lineas del xlsx referenciadas por actividad
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4g3Yf3jcPuX77QSmk15pC
</commit_message>
<xml_diff>
--- a/fovi2026/FOVI2026_Presupuesto-carta-gantt_v0.1.xlsx
+++ b/fovi2026/FOVI2026_Presupuesto-carta-gantt_v0.1.xlsx
@@ -2981,7 +2981,7 @@
       <c r="B27" s="192" t="n"/>
       <c r="C27" s="190" t="inlineStr">
         <is>
-          <t>3.3 Visita de investigadores IPC y UJPA: ponencias en Santiago y jornada en una región asociada</t>
+          <t>3.3 Visita de investigadores de Coimbra y UJPA: ponencias en Santiago</t>
         </is>
       </c>
       <c r="D27" s="191" t="inlineStr">
@@ -3019,7 +3019,7 @@
       <c r="B28" s="192" t="n"/>
       <c r="C28" s="190" t="inlineStr">
         <is>
-          <t>3.4 Taller presencial en Santiago con estudiantes, tesistas y equipos de salud</t>
+          <t>3.4 Taller presencial en Santiago y jornada territorial en una región asociada</t>
         </is>
       </c>
       <c r="D28" s="191" t="inlineStr">
@@ -5991,7 +5991,7 @@
       </c>
       <c r="D23" s="235" t="inlineStr">
         <is>
-          <t>Pasantía en Coimbra (ISEC-IPC, Portugal): 2 integrantes del grupo chileno (1 USACH, 1 UCM). 2 pasajes aéreos económicos Santiago–Coimbra (vía Lisboa/Porto), ida y vuelta, punto a punto, 2 × $1.500.000. ESTIMACIÓN: cotizar antes de enviar.</t>
+          <t>Actividad 5. Pasantía en Coimbra (ISEC-IPC, Portugal): 2 integrantes del grupo chileno (1 USACH, 1 UCM). 2 pasajes aéreos económicos Santiago–Coimbra (vía Lisboa/Porto), ida y vuelta, punto a punto, 2 × $1.500.000. ESTIMACIÓN: cotizar antes de enviar.</t>
         </is>
       </c>
       <c r="H23" s="231" t="n"/>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="D24" s="236" t="inlineStr">
         <is>
-          <t>Pasantía en Luanda (UJPA, Angola): 2 integrantes del grupo chileno (USACH y UCM). 2 pasajes aéreos económicos Santiago–Luanda, ida y vuelta, 2 × $2.500.000. ESTIMACIÓN: cotizar antes de enviar.</t>
+          <t>Actividad 6. Pasantía en Luanda (UJPA, Angola): 2 integrantes del grupo chileno (USACH y UCM). 2 pasajes aéreos económicos Santiago–Luanda, ida y vuelta, 2 × $2.500.000. ESTIMACIÓN: cotizar antes de enviar.</t>
         </is>
       </c>
       <c r="H24" s="231" t="n"/>
@@ -6039,7 +6039,7 @@
       </c>
       <c r="D25" s="236" t="inlineStr">
         <is>
-          <t>Seguro de viaje, pasantía Coimbra: 2 personas × $60.000. ESTIMACIÓN.</t>
+          <t>Actividad 5. Seguro de viaje, pasantía Coimbra: 2 personas × $60.000. ESTIMACIÓN.</t>
         </is>
       </c>
       <c r="H25" s="231" t="n"/>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="D26" s="236" t="inlineStr">
         <is>
-          <t>Seguro de viaje, pasantía Luanda: 2 personas × $60.000. ESTIMACIÓN.</t>
+          <t>Actividad 6. Seguro de viaje, pasantía Luanda: 2 personas × $60.000. ESTIMACIÓN.</t>
         </is>
       </c>
       <c r="H26" s="231" t="n"/>
@@ -6087,7 +6087,7 @@
       </c>
       <c r="D27" s="236" t="inlineStr">
         <is>
-          <t>Pasantía Coimbra: 2 personas × 7 días × $180.000 por día (tope de viático internacional: $250.000 por persona y día).</t>
+          <t>Actividad 5. Pasantía Coimbra: 2 personas × 7 días × $180.000 por día (tope de viático internacional: $250.000 por persona y día).</t>
         </is>
       </c>
       <c r="H27" s="231" t="n"/>
@@ -6111,7 +6111,7 @@
       </c>
       <c r="D28" s="236" t="inlineStr">
         <is>
-          <t>Pasantía Luanda: 2 personas × 8 días × $200.000 por día (tope: $250.000 por persona y día).</t>
+          <t>Actividad 6. Pasantía Luanda: 2 personas × 8 días × $200.000 por día (tope: $250.000 por persona y día).</t>
         </is>
       </c>
       <c r="H28" s="231" t="n"/>
@@ -6135,7 +6135,7 @@
       </c>
       <c r="D29" s="236" t="inlineStr">
         <is>
-          <t>Software SIG, datos y licencias para el protocolo común y el análisis geoespacial del estudio comparado (Santiago, regiones asociadas, Luanda, centro de Portugal). ESTIMACIÓN.</t>
+          <t>Actividad 4. Software SIG, datos y licencias para el protocolo común y el análisis geoespacial del estudio comparado (Santiago, regiones asociadas, Luanda, centro de Portugal). ESTIMACIÓN.</t>
         </is>
       </c>
       <c r="H29" s="231" t="n"/>
@@ -7739,7 +7739,7 @@
       </c>
       <c r="D20" s="235" t="inlineStr">
         <is>
-          <t>Visita a Chile de un/a investigador/a del IPC (Portugal) para ponencias y taller en Santiago y una región asociada: pasaje aéreo económico ida y vuelta. ESTIMACIÓN: cotizar.</t>
+          <t>Actividad 10. Visita a Chile de un/a investigador/a del IPC (Portugal) para ponencias y taller en Santiago y una región asociada: pasaje aéreo económico ida y vuelta. ESTIMACIÓN: cotizar.</t>
         </is>
       </c>
     </row>
@@ -7754,7 +7754,7 @@
       </c>
       <c r="D21" s="236" t="inlineStr">
         <is>
-          <t>Visita a Chile de un/a investigador/a de la UJPA (Angola): pasaje aéreo económico ida y vuelta. ESTIMACIÓN: cotizar.</t>
+          <t>Actividad 10. Visita a Chile de un/a investigador/a de la UJPA (Angola): pasaje aéreo económico ida y vuelta. ESTIMACIÓN: cotizar.</t>
         </is>
       </c>
     </row>
@@ -7769,7 +7769,7 @@
       </c>
       <c r="D22" s="236" t="inlineStr">
         <is>
-          <t>2 investigadores/as extranjeros/as × 8 días × $150.000 por día (tope de viático nacional $150.000/día; máximo 10 días). Alojamiento y manutención en Santiago y una región asociada.</t>
+          <t>Actividad 10. 2 investigadores/as extranjeros/as × 8 días × $150.000 por día (tope de viático nacional $150.000/día; máximo 10 días). Alojamiento y manutención en Santiago y una región asociada.</t>
         </is>
       </c>
     </row>
@@ -7784,7 +7784,7 @@
       </c>
       <c r="D23" s="236" t="inlineStr">
         <is>
-          <t>Seguro de viaje de los 2 investigadores/as extranjeros/as: 2 × $60.000. ESTIMACIÓN.</t>
+          <t>Actividad 10. Seguro de viaje de los 2 investigadores/as extranjeros/as: 2 × $60.000. ESTIMACIÓN.</t>
         </is>
       </c>
     </row>
@@ -7799,7 +7799,7 @@
       </c>
       <c r="D24" s="236" t="inlineStr">
         <is>
-          <t>Traslado terrestre a la región asociada (ida y vuelta) para la jornada territorial. ESTIMACIÓN: ajustar según destino (con Biobío probablemente sube).</t>
+          <t>Actividad 11. Traslado terrestre a la región asociada (ida y vuelta) para la jornada territorial. ESTIMACIÓN: ajustar según destino (con Biobío probablemente sube).</t>
         </is>
       </c>
     </row>
@@ -7814,7 +7814,7 @@
       </c>
       <c r="D25" s="236" t="inlineStr">
         <is>
-          <t>Tres seminarios virtuales bilingües español–portugués: plataforma de videoconferencia, transmisión en vivo e interpretación simultánea ES–PT (3 × $500.000). ESTIMACIÓN: cotizar.</t>
+          <t>Actividad 8, 9 y 12. Tres seminarios virtuales bilingües español–portugués: plataforma de videoconferencia, transmisión en vivo e interpretación simultánea ES–PT (3 × $500.000). ESTIMACIÓN: cotizar.</t>
         </is>
       </c>
     </row>
@@ -7829,7 +7829,7 @@
       </c>
       <c r="D26" s="236" t="inlineStr">
         <is>
-          <t>Taller presencial en Santiago y jornada territorial en una región asociada con las instituciones nacionales asociadas: arriendo de sala, materiales y difusión. No incluye alimentación ni honorarios de organización.</t>
+          <t>Actividad 11. Taller presencial en Santiago y jornada territorial en una región asociada con las instituciones nacionales asociadas: arriendo de sala, materiales y difusión. No incluye alimentación ni honorarios de organización.</t>
         </is>
       </c>
     </row>
@@ -7844,7 +7844,7 @@
       </c>
       <c r="D27" s="236" t="inlineStr">
         <is>
-          <t>Inscripción de integrantes del grupo chileno a un congreso para presentar resultados del estudio. ESTIMACIÓN.</t>
+          <t>Actividad 16. Inscripción de integrantes del grupo chileno a un congreso para presentar resultados del estudio. ESTIMACIÓN.</t>
         </is>
       </c>
     </row>
@@ -7859,7 +7859,7 @@
       </c>
       <c r="D28" s="236" t="inlineStr">
         <is>
-          <t>Diseño, traducción ES–PT y difusión del policy brief bilingüe. ESTIMACIÓN.</t>
+          <t>Actividad 13. Diseño, traducción ES–PT y difusión del policy brief bilingüe. ESTIMACIÓN.</t>
         </is>
       </c>
     </row>
@@ -7874,7 +7874,7 @@
       </c>
       <c r="D29" s="236" t="inlineStr">
         <is>
-          <t>Gastos de administración ligados a la gestión del proyecto. VERIFICAR en numeral 2.5.4 de las bases que sean financiables antes de enviar.</t>
+          <t>Actividad 3. Gastos de administración ligados a la gestión del proyecto. VERIFICAR en numeral 2.5.4 de las bases que sean financiables antes de enviar.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FOVI 2026: Universidade Politécnica de Coimbra en formulario v0.4 y presupuesto
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4g3Yf3jcPuX77QSmk15pC
</commit_message>
<xml_diff>
--- a/fovi2026/FOVI2026_Presupuesto-carta-gantt_v0.1.xlsx
+++ b/fovi2026/FOVI2026_Presupuesto-carta-gantt_v0.1.xlsx
@@ -2106,7 +2106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:Q102"/>
+  <dimension ref="A1:Q102"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15"/>
   <cols>
     <col width="2.7109375" customWidth="1" min="1" max="1"/>
@@ -2116,6 +2116,7 @@
     <col width="4.5703125" customWidth="1" min="6" max="17"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="39.75" customHeight="1">
       <c r="B2" s="182" t="inlineStr">
         <is>
@@ -2368,7 +2369,7 @@
     <row r="11">
       <c r="B11" s="189" t="inlineStr">
         <is>
-          <t>Objetivo 1 (OE1): Formalizar y activar la red USACH–UCM–UJPA–IPC–UNESPAR–UNILAB</t>
+          <t>Objetivo 1 (OE1): Formalizar y activar la red USACH–UCM–UJPA–UPCoimbra–UNESPAR–UNILAB</t>
         </is>
       </c>
       <c r="C11" s="190" t="inlineStr">
@@ -4603,7 +4604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I48"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="9.140625" customWidth="1" style="13" min="1" max="2"/>
@@ -5450,6 +5451,7 @@
       <c r="H42" s="34" t="n"/>
       <c r="I42" s="35" t="n"/>
     </row>
+    <row r="43"/>
     <row r="44" ht="15.75" customHeight="1">
       <c r="B44" s="36" t="inlineStr">
         <is>
@@ -5529,7 +5531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:S82"/>
+  <dimension ref="A1:S82"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="11.42578125" customWidth="1" style="76" min="1" max="1"/>
@@ -5542,6 +5544,7 @@
     <col width="11.42578125" customWidth="1" style="76" min="8" max="14"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="80" t="inlineStr">
         <is>
@@ -5549,6 +5552,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="80" t="inlineStr">
         <is>
@@ -5991,7 +5995,7 @@
       </c>
       <c r="D23" s="235" t="inlineStr">
         <is>
-          <t>Actividad 5. Pasantía en Coimbra (ISEC-IPC, Portugal): 2 integrantes del grupo chileno (1 USACH, 1 UCM). 2 pasajes aéreos económicos Santiago–Coimbra (vía Lisboa/Porto), ida y vuelta, punto a punto, 2 × $1.500.000. ESTIMACIÓN: cotizar antes de enviar.</t>
+          <t>Actividad 5. Pasantía en Coimbra (ISEC-UPCoimbra, Portugal): 2 integrantes del grupo chileno (1 USACH, 1 UCM). 2 pasajes aéreos económicos Santiago–Coimbra (vía Lisboa/Porto), ida y vuelta, punto a punto, 2 × $1.500.000. ESTIMACIÓN: cotizar antes de enviar.</t>
         </is>
       </c>
       <c r="H23" s="231" t="n"/>
@@ -6552,7 +6556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:S84"/>
+  <dimension ref="A1:S84"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="29.42578125" customWidth="1" min="2" max="2"/>
@@ -6562,6 +6566,7 @@
     <col width="10" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="49" t="inlineStr">
         <is>
@@ -6569,6 +6574,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="80" t="inlineStr">
         <is>
@@ -7428,7 +7434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:S79"/>
+  <dimension ref="A1:S79"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="29.42578125" customWidth="1" min="2" max="2"/>
@@ -7437,6 +7443,7 @@
     <col width="21.140625" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="49" t="inlineStr">
         <is>
@@ -7444,6 +7451,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="80" t="inlineStr">
         <is>
@@ -7739,7 +7747,7 @@
       </c>
       <c r="D20" s="235" t="inlineStr">
         <is>
-          <t>Actividad 10. Visita a Chile de un/a investigador/a del IPC (Portugal) para ponencias y taller en Santiago y una región asociada: pasaje aéreo económico ida y vuelta. ESTIMACIÓN: cotizar.</t>
+          <t>Actividad 10. Visita a Chile de un/a investigador/a de la UPCoimbra (Portugal) para ponencias y taller en Santiago y una región asociada: pasaje aéreo económico ida y vuelta. ESTIMACIÓN: cotizar.</t>
         </is>
       </c>
     </row>
@@ -8251,7 +8259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:E32"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="11.42578125" customWidth="1" min="1" max="1"/>
@@ -8261,6 +8269,7 @@
     <col width="25" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="32.25" customHeight="1">
       <c r="B2" s="181" t="inlineStr">
         <is>

</xml_diff>